<commit_message>
alv ya me quiero dormir
</commit_message>
<xml_diff>
--- a/TAREAS 6 SEMESTRE/Aprendizaje Machín/EvaluaciónModelos+Métricas.xlsx
+++ b/TAREAS 6 SEMESTRE/Aprendizaje Machín/EvaluaciónModelos+Métricas.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vmvic\Desktop\CUCEI\TAREAS 6 SEMESTRE\Aprendizaje Machín\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84F71A89-4BA5-42C7-BBAF-83ECE6BB1BE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DDB302F-1D0B-4DBA-9C48-B606CDFFCF14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{EA3FA98A-E78B-4AEF-B769-394AFD4A17D1}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{EA3FA98A-E78B-4AEF-B769-394AFD4A17D1}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="19">
   <si>
     <t>Evaluación de modelos</t>
   </si>
@@ -72,6 +72,30 @@
   </si>
   <si>
     <t>Total</t>
+  </si>
+  <si>
+    <t>Clase A</t>
+  </si>
+  <si>
+    <t>Rendimiento General del Modelo</t>
+  </si>
+  <si>
+    <t>Clase B</t>
+  </si>
+  <si>
+    <t>Clase C</t>
+  </si>
+  <si>
+    <t>Clase D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Presición </t>
+  </si>
+  <si>
+    <t xml:space="preserve">F1-Score </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Especifidad </t>
   </si>
 </sst>
 </file>
@@ -87,12 +111,30 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="5">
@@ -159,19 +201,38 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -192,7 +253,7 @@
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Amarillo">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -200,34 +261,34 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="0E2841"/>
+        <a:srgbClr val="39302A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E8E8E8"/>
+        <a:srgbClr val="E5DEDB"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="156082"/>
+        <a:srgbClr val="FFCA08"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="E97132"/>
+        <a:srgbClr val="F8931D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="196B24"/>
+        <a:srgbClr val="CE8D3E"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="0F9ED5"/>
+        <a:srgbClr val="EC7016"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="A02B93"/>
+        <a:srgbClr val="E64823"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="4EA72E"/>
+        <a:srgbClr val="9C6A6A"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="467886"/>
+        <a:srgbClr val="2998E3"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="96607D"/>
+        <a:srgbClr val="7F723D"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -506,99 +567,417 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B6FE71E-19E5-4EFF-AEA8-CA00AE9EFF87}">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:S15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="12.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
       <c r="D1" s="4"/>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="F1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="4"/>
+      <c r="K1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="L1" s="3"/>
+      <c r="M1" s="3"/>
+      <c r="N1" s="4"/>
+      <c r="P1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="Q1" s="3"/>
+      <c r="R1" s="3"/>
+      <c r="S1" s="4"/>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="8"/>
+      <c r="F2" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" s="7"/>
+      <c r="H2" s="7"/>
+      <c r="I2" s="8"/>
+      <c r="K2" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="L2" s="7"/>
+      <c r="M2" s="7"/>
+      <c r="N2" s="8"/>
+      <c r="P2" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q2" s="7"/>
+      <c r="R2" s="7"/>
+      <c r="S2" s="8"/>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="1">
+      <c r="B3" s="1">
         <v>8</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C3" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="1">
-        <f>B2/(B2+B4)</f>
+      <c r="D3" s="1">
+        <f>B3/(B3+B5)</f>
         <v>0.8</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="F3" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="G3" s="1">
+        <v>7</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="I3" s="1">
+        <f>G3/(G3+G5)</f>
+        <v>0.7</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="L3" s="1">
+        <v>7</v>
+      </c>
+      <c r="M3" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="N3" s="1">
+        <f>L3/(L3+L5)</f>
+        <v>0.63636363636363635</v>
+      </c>
+      <c r="P3" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q3" s="1">
+        <v>7</v>
+      </c>
+      <c r="R3" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="S3" s="1">
+        <f>Q3/(Q3+Q5)</f>
+        <v>0.77777777777777779</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
         <v>3</v>
-      </c>
-      <c r="B3" s="1">
-        <v>2</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D3" s="1">
-        <f>2*((D2*D4)/(D2+D4))</f>
-        <v>0.80000000000000016</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>2</v>
       </c>
       <c r="B4" s="1">
         <v>2</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" s="1">
+        <f>2*((D3*D5)/(D3+D5))</f>
+        <v>0.80000000000000016</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G4" s="1">
+        <v>3</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="I4" s="1">
+        <f>2*((I3*I5)/(I3+I5))</f>
+        <v>0.7</v>
+      </c>
+      <c r="K4" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="L4" s="1">
+        <v>3</v>
+      </c>
+      <c r="M4" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="N4" s="1">
+        <f>2*((N3*N5)/(N3+N5))</f>
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="P4" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q4" s="1">
+        <v>3</v>
+      </c>
+      <c r="R4" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="S4" s="1">
+        <f>2*((S3*S5)/(S3+S5))</f>
+        <v>0.73684210526315774</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="1">
+        <v>2</v>
+      </c>
+      <c r="C5" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="1">
-        <f>B2/(B2+B3)</f>
+      <c r="D5" s="1">
+        <f>B3/(B3+B4)</f>
         <v>0.8</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="F5" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="G5" s="1">
+        <v>3</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="I5" s="1">
+        <f>G3/(G3+G4)</f>
+        <v>0.7</v>
+      </c>
+      <c r="K5" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="L5" s="1">
         <v>4</v>
       </c>
-      <c r="B5" s="1">
+      <c r="M5" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="N5" s="1">
+        <f>L3/(L3+L4)</f>
+        <v>0.7</v>
+      </c>
+      <c r="P5" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="Q5" s="1">
+        <v>2</v>
+      </c>
+      <c r="R5" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="S5" s="1">
+        <f>Q3/(Q3+Q4)</f>
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="1">
         <v>28</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C6" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="1">
-        <f>B5/(B5+B4)</f>
+      <c r="D6" s="1">
+        <f>B6/(B6+B5)</f>
         <v>0.93333333333333335</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
+      <c r="F6" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="G6" s="1">
+        <v>27</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="I6" s="1">
+        <f>G6/(G6+G5)</f>
+        <v>0.9</v>
+      </c>
+      <c r="K6" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="L6" s="1">
+        <v>26</v>
+      </c>
+      <c r="M6" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="N6" s="1">
+        <f>L6/(L6+L5)</f>
+        <v>0.8666666666666667</v>
+      </c>
+      <c r="P6" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="Q6" s="1">
+        <v>28</v>
+      </c>
+      <c r="R6" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="S6" s="1">
+        <f>Q6/(Q6+Q5)</f>
+        <v>0.93333333333333335</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="1">
-        <f>B2+B3+B4+B5</f>
+      <c r="B7" s="1">
+        <f>B3+B4+B5+B6</f>
         <v>40</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C7" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="1">
-        <f>(B2+B5)/(B2+B3+B4+B5)</f>
+      <c r="D7" s="1">
+        <f>(B3+B6)/(B3+B4+B5+B6)</f>
         <v>0.9</v>
       </c>
+      <c r="F7" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G7" s="1">
+        <f>G3+G4+G5+G6</f>
+        <v>40</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="I7" s="1">
+        <f>(G3+G6)/(G3+G4+G5+G6)</f>
+        <v>0.85</v>
+      </c>
+      <c r="K7" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="L7" s="1">
+        <f>L3+L4+L5+L6</f>
+        <v>40</v>
+      </c>
+      <c r="M7" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="N7" s="1">
+        <f>(L3+L6)/(L3+L4+L5+L6)</f>
+        <v>0.82499999999999996</v>
+      </c>
+      <c r="P7" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q7" s="1">
+        <f>Q3+Q4+Q5+Q6</f>
+        <v>40</v>
+      </c>
+      <c r="R7" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="S7" s="1">
+        <f>(Q3+Q6)/(Q3+Q4+Q5+Q6)</f>
+        <v>0.875</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="9"/>
+    </row>
+    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A11" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" s="12"/>
+      <c r="C11" s="11"/>
+      <c r="D11" s="1">
+        <f>(D3+I3+N3+S3)/4</f>
+        <v>0.72853535353535348</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A12" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" s="12"/>
+      <c r="C12" s="11"/>
+      <c r="D12" s="1">
+        <f t="shared" ref="D12:D15" si="0">(D4+I4+N4+S4)/4</f>
+        <v>0.72587719298245612</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A13" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="B13" s="12"/>
+      <c r="C13" s="11"/>
+      <c r="D13" s="1">
+        <f t="shared" si="0"/>
+        <v>0.72500000000000009</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A14" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" s="12"/>
+      <c r="C14" s="11"/>
+      <c r="D14" s="1">
+        <f t="shared" si="0"/>
+        <v>0.90833333333333344</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A15" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B15" s="12"/>
+      <c r="C15" s="11"/>
+      <c r="D15" s="1">
+        <f t="shared" si="0"/>
+        <v>0.86250000000000004</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="14">
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="K1:N1"/>
+    <mergeCell ref="K2:N2"/>
+    <mergeCell ref="P1:S1"/>
+    <mergeCell ref="P2:S2"/>
+    <mergeCell ref="A10:C10"/>
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="F1:I1"/>
+    <mergeCell ref="F2:I2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>